<commit_message>
Session 111b: the >=50% subset rests on state award sources only; Rhode Island out (owner decision)
A state with any award row from CMS's Obligated Funds Report is left out of
US_GE50 whatever its share (RI, 50.4% on CMS lines alone, today; NE and PA
would be left out whole if they crossed). The builder refuses if a
CMS-obligation dollar reaches the row. Label, Definitions and the Notes
entry state the criterion.

21 states: allotment $4,284,392,337; awards $3,362,841,950.78; hospital best
estimate $1,557,146,269.69 (46.3% of awards, 36.3% of allotment); strict
named $1,451,104,633.38 (unchanged: RI has no named-hospital dollars).
Re-pinned in test_08; the first 51 CSV rows are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1P5eQVRZaY3QTvr6BikAp
</commit_message>
<xml_diff>
--- a/output/year1_summary_2026-10-29.xlsx
+++ b/output/year1_summary_2026-10-29.xlsx
@@ -219,7 +219,7 @@
     <t xml:space="preserve">4 Complete of 50</t>
   </si>
   <si>
-    <t xml:space="preserve">States with ≥50% published (n = 22)</t>
+    <t xml:space="preserve">States with ≥50% published, state award sources (n = 21)</t>
   </si>
   <si>
     <t xml:space="preserve">n/m</t>
@@ -516,7 +516,7 @@
     <t xml:space="preserve">US_GE50</t>
   </si>
   <si>
-    <t xml:space="preserve">4 COMPLETE of 22: AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR RI SC SD TX VT WY</t>
+    <t xml:space="preserve">4 COMPLETE of 21: AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR SC SD TX VT WY</t>
   </si>
   <si>
     <t xml:space="preserve">sheet</t>
@@ -531,7 +531,7 @@
     <t xml:space="preserve">Overview</t>
   </si>
   <si>
-    <t xml:space="preserve">State name. Below the 50 states: the national total (the sum of the 50 state rows), then the states whose awards published are at least 50% of their allotment (n in the label), which shows only allotment, awards published, the hospital figures and strict named-hospital dollars. The second row is a subset of the national total, never added to it.</t>
+    <t xml:space="preserve">State name. Below the 50 states: the national total (the sum of the 50 state rows), then the states whose awards published are at least 50% of their allotment and rest on state award sources only (n in the label; a state with any CMS obligation-report row is left out), which shows only allotment, awards published, the hospital figures and strict named-hospital dollars. The second row is a subset of the national total, never added to it.</t>
   </si>
   <si>
     <t xml:space="preserve">Plain-language Year 1 status; each label is defined below.</t>
@@ -582,7 +582,7 @@
     <t xml:space="preserve">Detail</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-letter state code. US is the national row (the sum of the 50 state rows). US_GE50 is the second national row: the sum over the states whose awards published are at least 50% of their allotment (a subset of US, never added to it).</t>
+    <t xml:space="preserve">Two-letter state code. US is the national row (the sum of the 50 state rows). US_GE50 is the second national row: the sum over the states whose awards published are at least 50% of their allotment AND rest on state award sources only (a state with any CMS obligation-report row, such as Rhode Island, is left out); a subset of US, never added to it.</t>
   </si>
   <si>
     <t xml:space="preserve">State name.</t>
@@ -735,7 +735,7 @@
     <t xml:space="preserve">n/m (HOSPITAL % OF AWARDS). Shown only where awards published are at least 50% of the allotment. Not meaningful where most of the state's money is not yet published; e.g., Illinois's only published award is ICAHN's hospital network grant. The national hospital share of awards is reported only for states where most of the money is published (see the second national row). Hospital % of allotment is shown for every state.</t>
   </si>
   <si>
-    <t xml:space="preserve">SECOND NATIONAL ROW. 'States with ≥50% published (n = 22)' sums the states whose awards published are at least 50% of their allotment (AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR RI SC SD TX VT WY): allotment $4,440,562,268, awards published $3,441,569,061, hospital best estimate $1,572,986,177 (45.7% of those awards). It is a subset of the national row, never added to it. Rhode Island qualifies on CMS obligation-report lines alone; the set changes as states publish.</t>
+    <t xml:space="preserve">SECOND NATIONAL ROW. 'States with ≥50% published, state award sources (n = 21)' sums the states whose awards published are at least 50% of their allotment AND rest on state award sources only: a state with any award row taken from CMS's Obligated Funds Report is left out, whatever its share (excluded today: Rhode Island (50.4%, CMS obligation lines)). Members (AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR SC SD TX VT WY): allotment $4,284,392,337, awards published $3,362,841,951, hospital best estimate $1,557,146,270 (46.3% of those awards). It is a subset of the national row, never added to it; the set changes as states publish.</t>
   </si>
   <si>
     <t xml:space="preserve">CONFIDENTIAL SOURCES. Figures or rows flagged here rest on, or cite, Delaware's confidential source (DE Verify.xlsx). They must not leave the team. As built, no award row or figure cites it; Delaware's status-table notes do (confidential_source_flag; the row is shaded on Overview and Detail).</t>
@@ -1900,7 +1900,7 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="38.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="59.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="31.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="19.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="19.71" hidden="0" customWidth="1"/>
@@ -3582,20 +3582,20 @@
       </c>
       <c r="B53" s="8"/>
       <c r="C53" s="5" t="n">
-        <v>4440562268</v>
+        <v>4284392337</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>3441569061.22</v>
+        <v>3362841950.78</v>
       </c>
       <c r="E53" s="6"/>
       <c r="F53" s="5" t="n">
-        <v>1572986177.36</v>
+        <v>1557146269.69</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>0.45705495062836</v>
+        <v>0.463044737897606</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>0.354231307304348</v>
+        <v>0.363446236294116</v>
       </c>
       <c r="I53" s="5" t="n">
         <v>1451104633.38</v>
@@ -3614,7 +3614,7 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="10.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="38.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="59.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="60.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="18.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
@@ -9539,37 +9539,37 @@
         <v>166</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>4440562268</v>
+        <v>4284392337</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>3441</v>
+        <v>3337</v>
       </c>
       <c r="G53" s="8" t="n">
-        <v>3125</v>
+        <v>3021</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>3028965541.22</v>
+        <v>2950238430.78</v>
       </c>
       <c r="I53" s="5" t="n">
         <v>412603520</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>3441569061.22</v>
+        <v>3362841950.78</v>
       </c>
       <c r="K53" s="6" t="n">
-        <v>0.775030019513736</v>
+        <v>0.784905229555778</v>
       </c>
       <c r="L53" s="5" t="n">
         <v>1385478477.61</v>
       </c>
       <c r="M53" s="8" t="n">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="N53" s="5" t="n">
-        <v>1446728679.7</v>
+        <v>1430888772.03</v>
       </c>
       <c r="O53" s="5" t="n">
         <v>126257497.66</v>
@@ -9584,16 +9584,16 @@
         <v>0</v>
       </c>
       <c r="S53" s="8" t="n">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="T53" s="5" t="n">
-        <v>1572986177.36</v>
+        <v>1557146269.69</v>
       </c>
       <c r="U53" s="6" t="n">
-        <v>0.45705495062836</v>
+        <v>0.463044737897606</v>
       </c>
       <c r="V53" s="6" t="n">
-        <v>0.354231307304348</v>
+        <v>0.363446236294116</v>
       </c>
       <c r="W53" s="5" t="n">
         <v>1451104633.38</v>
@@ -9602,25 +9602,25 @@
         <v>54748315.31</v>
       </c>
       <c r="Y53" s="5" t="n">
-        <v>15839907.67</v>
+        <v>0</v>
       </c>
       <c r="Z53" s="5" t="n">
         <v>710051173.87</v>
       </c>
       <c r="AA53" s="5" t="n">
-        <v>52746543.98</v>
+        <v>36906636.31</v>
       </c>
       <c r="AB53" s="5" t="n">
-        <v>15839907.67</v>
+        <v>0</v>
       </c>
       <c r="AC53" s="5" t="n">
         <v>55305273.31</v>
       </c>
       <c r="AD53" s="5" t="n">
-        <v>126762455.53</v>
+        <v>110922547.86</v>
       </c>
       <c r="AE53" s="5" t="n">
-        <v>253328337.11</v>
+        <v>237488429.44</v>
       </c>
       <c r="AF53" s="5" t="n">
         <v>512424850.1</v>

</xml_diff>

<commit_message>
Session 111b: subset rule on state-sourced awards (owner decision)
US_GE50 now drops the CMS obligation-report files (NE_CMS, PA_CMS, RI)
and rebuilds the state table without them, so each state's "% published" is
its state-sourced award total over its allotment and a state qualifies at
>=50%. A state with CMS lines keeps its state-sourced dollars. The builder
still refuses any CMS-obligation dollar in the row, and now also refuses an
award file mixing CMS lines with state-sourced rows. Notes and Definitions
state the rule and each CMS-line state's share both ways (RI 0.0% vs 50.4%,
NE 19.1% vs 20.9%, PA 21.8% vs 23.4%).

Today's 21-state row is unchanged: the CSV is byte-identical. test_08 adds
the state-sourced table checks and drives both guards.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1P5eQVRZaY3QTvr6BikAp
</commit_message>
<xml_diff>
--- a/output/year1_summary_2026-10-29.xlsx
+++ b/output/year1_summary_2026-10-29.xlsx
@@ -531,7 +531,7 @@
     <t xml:space="preserve">Overview</t>
   </si>
   <si>
-    <t xml:space="preserve">State name. Below the 50 states: the national total (the sum of the 50 state rows), then the states whose awards published are at least 50% of their allotment and rest on state award sources only (n in the label; a state with any CMS obligation-report row is left out), which shows only allotment, awards published, the hospital figures and strict named-hospital dollars. The second row is a subset of the national total, never added to it.</t>
+    <t xml:space="preserve">State name. Below the 50 states: the national total (the sum of the 50 state rows), then the states whose state-sourced awards published are at least 50% of their allotment (n in the label; CMS obligation-report rows are removed from that row's figures and from each state's test), which shows only allotment, awards published, the hospital figures and strict named-hospital dollars. The second row is a subset of the national total, never added to it.</t>
   </si>
   <si>
     <t xml:space="preserve">Plain-language Year 1 status; each label is defined below.</t>
@@ -582,7 +582,7 @@
     <t xml:space="preserve">Detail</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-letter state code. US is the national row (the sum of the 50 state rows). US_GE50 is the second national row: the sum over the states whose awards published are at least 50% of their allotment AND rest on state award sources only (a state with any CMS obligation-report row, such as Rhode Island, is left out); a subset of US, never added to it.</t>
+    <t xml:space="preserve">Two-letter state code. US is the national row (the sum of the 50 state rows). US_GE50 is the second national row, on state award sources only: CMS obligation-report rows are removed from all its figures, and it sums the states whose state-sourced awards published are at least 50% of their allotment (Rhode Island, whose only rows are CMS lines, cannot qualify); a subset of US, never added to it.</t>
   </si>
   <si>
     <t xml:space="preserve">State name.</t>
@@ -735,7 +735,7 @@
     <t xml:space="preserve">n/m (HOSPITAL % OF AWARDS). Shown only where awards published are at least 50% of the allotment. Not meaningful where most of the state's money is not yet published; e.g., Illinois's only published award is ICAHN's hospital network grant. The national hospital share of awards is reported only for states where most of the money is published (see the second national row). Hospital % of allotment is shown for every state.</t>
   </si>
   <si>
-    <t xml:space="preserve">SECOND NATIONAL ROW. 'States with ≥50% published, state award sources (n = 21)' sums the states whose awards published are at least 50% of their allotment AND rest on state award sources only: a state with any award row taken from CMS's Obligated Funds Report is left out, whatever its share (excluded today: Rhode Island (50.4%, CMS obligation lines)). Members (AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR SC SD TX VT WY): allotment $4,284,392,337, awards published $3,362,841,951, hospital best estimate $1,557,146,270 (46.3% of those awards). It is a subset of the national row, never added to it; the set changes as states publish.</t>
+    <t xml:space="preserve">SECOND NATIONAL ROW. 'States with ≥50% published, state award sources (n = 21)' rests on state award sources only. Rows taken from CMS's Obligated Funds Report are removed from every figure in it, each state's '% published' is computed on its state-sourced awards alone, and a state qualifies when those are at least 50% of its allotment. States carrying CMS obligation lines today: Nebraska 19.1% state-sourced (20.9% with CMS lines; does not qualify); Pennsylvania 21.8% state-sourced (23.4% with CMS lines; does not qualify); Rhode Island 0.0% state-sourced (50.4% with CMS lines; does not qualify). Members (AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR SC SD TX VT WY): allotment $4,284,392,337, awards published $3,362,841,951, hospital best estimate $1,557,146,270 (46.3% of those awards). It is a subset of the national row, never added to it; the set changes as states publish.</t>
   </si>
   <si>
     <t xml:space="preserve">CONFIDENTIAL SOURCES. Figures or rows flagged here rest on, or cite, Delaware's confidential source (DE Verify.xlsx). They must not leave the team. As built, no award row or figure cites it; Delaware's status-table notes do (confidential_source_flag; the row is shaded on Overview and Detail).</t>

</xml_diff>

<commit_message>
Session 111b: state rows' n/m test on state-sourced awards (owner decision)
Hospital % of awards now reads n/m wherever a state's STATE-SOURCED awards
(CMS obligation-report files removed, as for the second national row) are
under 50% of its allotment. Rhode Island (0.0% state-sourced, 50.4% with CMS
lines) becomes n/m on Overview and Detail; a cell-by-cell diff of the
workbook shows no other figure moved. 29 states and the national row read
n/m. The CSV is unchanged and keeps every computed share. Definitions and
the n/m note state the rule; test_08 pins that RI is the only state the test
moved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1P5eQVRZaY3QTvr6BikAp
</commit_message>
<xml_diff>
--- a/output/year1_summary_2026-10-29.xlsx
+++ b/output/year1_summary_2026-10-29.xlsx
@@ -549,7 +549,7 @@
     <t xml:space="preserve">BEST ESTIMATE of Year 1 RHTP dollars reaching hospitals: source-coded plus best-judgment hospital dollars (Detail: hospital_summary_usd).</t>
   </si>
   <si>
-    <t xml:space="preserve">Best-estimate hospital dollars as a share of awards published. Shown only where awards published are at least 50% of the allotment; otherwise n/m (not meaningful) (Detail: hospital_share_of_awards_pct).</t>
+    <t xml:space="preserve">Best-estimate hospital dollars as a share of awards published. Shown only where the state's STATE-SOURCED awards published (CMS obligation-report rows left out) are at least 50% of its allotment; otherwise n/m (not meaningful) (Detail: hospital_share_of_awards_pct).</t>
   </si>
   <si>
     <t xml:space="preserve">Best-estimate hospital dollars as a share of the allotment, shown for every state (Detail: hospital_share_of_allotment_pct).</t>
@@ -642,7 +642,7 @@
     <t xml:space="preserve">BEST ESTIMATE of Year 1 RHTP dollars reaching hospitals: coded plus best-judgment hospital dollars.</t>
   </si>
   <si>
-    <t xml:space="preserve">Best-estimate hospital dollars as a percent of the published award total.</t>
+    <t xml:space="preserve">Best-estimate hospital dollars as a percent of the published award total. On the workbook's Detail sheet it reads n/m where the state's state-sourced awards (CMS obligation-report rows left out) are under 50% of its allotment; this CSV keeps the computed value.</t>
   </si>
   <si>
     <t xml:space="preserve">Best-estimate hospital dollars as a percent of the allotment.</t>
@@ -732,7 +732,7 @@
     <t xml:space="preserve">AWARD COVERAGE VARIES WIDELY BY STATE. Awards published run from 0% to 97.6% of the allotment, so a state's hospital share describes only the money that state has published so far. State shares are not comparable to one another.</t>
   </si>
   <si>
-    <t xml:space="preserve">n/m (HOSPITAL % OF AWARDS). Shown only where awards published are at least 50% of the allotment. Not meaningful where most of the state's money is not yet published; e.g., Illinois's only published award is ICAHN's hospital network grant. The national hospital share of awards is reported only for states where most of the money is published (see the second national row). Hospital % of allotment is shown for every state.</t>
+    <t xml:space="preserve">n/m (HOSPITAL % OF AWARDS). Shown only where the state's STATE-SOURCED awards published are at least 50% of its allotment: rows taken from CMS's Obligated Funds Report do not count toward the test, the same rule as the second national row (Rhode Island, whose only rows are CMS lines, reads n/m). Not meaningful where most of the state's money is not yet published; e.g., Illinois's only published award is ICAHN's hospital network grant. The national hospital share of awards is reported only for states where most of the money is published (see the second national row). Hospital % of allotment is shown for every state.</t>
   </si>
   <si>
     <t xml:space="preserve">SECOND NATIONAL ROW. 'States with ≥50% published, state award sources (n = 21)' rests on state award sources only. Rows taken from CMS's Obligated Funds Report are removed from every figure in it, each state's '% published' is computed on its state-sourced awards alone, and a state qualifies when those are at least 50% of its allotment. States carrying CMS obligation lines today: Nebraska 19.1% state-sourced (20.9% with CMS lines; does not qualify); Pennsylvania 21.8% state-sourced (23.4% with CMS lines; does not qualify); Rhode Island 0.0% state-sourced (50.4% with CMS lines; does not qualify). Members (AK AL AR CA CO FL GA ID IN MD MI MS NJ NV OH OR SC SD TX VT WY): allotment $4,284,392,337, awards published $3,362,841,951, hospital best estimate $1,557,146,270 (46.3% of those awards). It is a subset of the national row, never added to it; the set changes as states publish.</t>
@@ -3179,8 +3179,8 @@
       <c r="F40" s="2" t="n">
         <v>15839907.67</v>
       </c>
-      <c r="G40" s="3" t="n">
-        <v>0.20120016575576</v>
+      <c r="G40" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="H40" s="3" t="n">
         <v>0.101427384699299</v>
@@ -8120,8 +8120,8 @@
       <c r="T40" s="2" t="n">
         <v>15839907.67</v>
       </c>
-      <c r="U40" s="3" t="n">
-        <v>0.20120016575576</v>
+      <c r="U40" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="V40" s="3" t="n">
         <v>0.101427384699299</v>

</xml_diff>